<commit_message>
Adjust linear schedule for 5 staff March-June
Co-authored-by: asd111-oss <asd111-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/linear_schedule.xlsx
+++ b/linear_schedule.xlsx
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -89,6 +89,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,82 +458,142 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="20" max="20"/>
+    <col width="9" customWidth="1" min="21" max="21"/>
+    <col width="9" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Этап работ</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Начало</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>Окончание</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Длит., нед</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Н1</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Н2</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Н3</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Н4</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Н5</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Н6</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Н7</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Н8</t>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Кол-во сотрудников</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Март W1</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Март W2</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>Март W3</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Март W4</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Март W5</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Апрель W1</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Апрель W2</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Апрель W3</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Апрель W4</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Май W1</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>Май W2</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>Май W3</t>
+        </is>
+      </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>Май W4</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>Июнь W1</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>Июнь W2</t>
+        </is>
+      </c>
+      <c r="U1" s="5" t="inlineStr">
+        <is>
+          <t>Июнь W3</t>
+        </is>
+      </c>
+      <c r="V1" s="5" t="inlineStr">
+        <is>
+          <t>Июнь W4</t>
         </is>
       </c>
     </row>
@@ -542,109 +605,149 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>01.05.2026</t>
+          <t>01.03.2026</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>14.05.2026</t>
+          <t>14.03.2026</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
+      <c r="E2" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
           <t>██</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="H2" s="3" t="inlineStr"/>
       <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr"/>
       <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr"/>
+      <c r="M2" s="3" t="inlineStr"/>
+      <c r="N2" s="3" t="inlineStr"/>
+      <c r="O2" s="3" t="inlineStr"/>
+      <c r="P2" s="3" t="inlineStr"/>
+      <c r="Q2" s="3" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr"/>
+      <c r="S2" s="3" t="inlineStr"/>
+      <c r="T2" s="3" t="inlineStr"/>
+      <c r="U2" s="3" t="inlineStr"/>
+      <c r="V2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Земляные работы и основание</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>15.05.2026</t>
+          <t>15.03.2026</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>28.05.2026</t>
+          <t>04.04.2026</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
       <c r="K3" s="3" t="inlineStr"/>
       <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="3" t="inlineStr"/>
+      <c r="O3" s="3" t="inlineStr"/>
+      <c r="P3" s="3" t="inlineStr"/>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" s="3" t="inlineStr"/>
+      <c r="S3" s="3" t="inlineStr"/>
+      <c r="T3" s="3" t="inlineStr"/>
+      <c r="U3" s="3" t="inlineStr"/>
+      <c r="V3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Фундамент</t>
+          <t>Устройство фундамента</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>29.05.2026</t>
+          <t>05.04.2026</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>18.06.2026</t>
+          <t>25.04.2026</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr"/>
+      <c r="O4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="R4" s="3" t="inlineStr"/>
+      <c r="S4" s="3" t="inlineStr"/>
+      <c r="T4" s="3" t="inlineStr"/>
+      <c r="U4" s="3" t="inlineStr"/>
+      <c r="V4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -654,37 +757,53 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>19.06.2026</t>
+          <t>26.04.2026</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>09.07.2026</t>
+          <t>23.05.2026</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="inlineStr"/>
       <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+      <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="R5" s="3" t="inlineStr"/>
+      <c r="S5" s="3" t="inlineStr"/>
+      <c r="T5" s="3" t="inlineStr"/>
+      <c r="U5" s="3" t="inlineStr"/>
+      <c r="V5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -694,65 +813,93 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>10.07.2026</t>
+          <t>24.05.2026</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>23.07.2026</t>
+          <t>13.06.2026</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="F6" s="3" t="inlineStr"/>
       <c r="G6" s="3" t="inlineStr"/>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
+      <c r="J6" s="3" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="3" t="inlineStr"/>
+      <c r="O6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="U6" s="3" t="inlineStr"/>
+      <c r="V6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Внутренние инженерные сети</t>
+          <t>Инженерные сети</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>17.07.2026</t>
+          <t>14.06.2026</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>06.08.2026</t>
+          <t>27.06.2026</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="F7" s="3" t="inlineStr"/>
       <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="3" t="inlineStr"/>
+      <c r="O7" s="3" t="inlineStr"/>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr"/>
+      <c r="R7" s="3" t="inlineStr"/>
+      <c r="S7" s="3" t="inlineStr"/>
+      <c r="T7" s="3" t="inlineStr"/>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
         <is>
           <t>██</t>
         </is>
@@ -761,34 +908,46 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Отделочные работы</t>
+          <t>Отделочные работы и сдача</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>24.07.2026</t>
+          <t>21.06.2026</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>20.08.2026</t>
+          <t>30.06.2026</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>5</v>
+      </c>
       <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>██</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="3" t="inlineStr"/>
+      <c r="N8" s="3" t="inlineStr"/>
+      <c r="O8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr"/>
+      <c r="R8" s="3" t="inlineStr"/>
+      <c r="S8" s="3" t="inlineStr"/>
+      <c r="T8" s="3" t="inlineStr"/>
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>██</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
         <is>
           <t>██</t>
         </is>

</xml_diff>

<commit_message>
Account for holidays and add color legend in schedule
Co-authored-by: asd111-oss <asd111-oss@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/linear_schedule.xlsx
+++ b/linear_schedule.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,14 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +72,12 @@
         <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E06666"/>
+        <bgColor rgb="00E06666"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -93,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -119,6 +131,16 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -484,13 +506,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DW9"/>
+  <dimension ref="A1:DW16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="4.2" customWidth="1" min="6" max="6"/>
     <col width="4.2" customWidth="1" min="7" max="7"/>
@@ -634,7 +656,7 @@
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>Длит., дн</t>
+          <t>Длит., раб.дн</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
@@ -677,7 +699,7 @@
           <t>07.03</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>08.03</t>
         </is>
@@ -947,7 +969,7 @@
           <t>30.04</t>
         </is>
       </c>
-      <c r="BO1" s="6" t="inlineStr">
+      <c r="BO1" s="9" t="inlineStr">
         <is>
           <t>01.05</t>
         </is>
@@ -987,7 +1009,7 @@
           <t>08.05</t>
         </is>
       </c>
-      <c r="BW1" s="6" t="inlineStr">
+      <c r="BW1" s="9" t="inlineStr">
         <is>
           <t>09.05</t>
         </is>
@@ -1157,7 +1179,7 @@
           <t>11.06</t>
         </is>
       </c>
-      <c r="DE1" s="6" t="inlineStr">
+      <c r="DE1" s="9" t="inlineStr">
         <is>
           <t>12.06</t>
         </is>
@@ -1294,7 +1316,7 @@
           <t>Сб</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>Вс</t>
         </is>
@@ -1564,7 +1586,7 @@
           <t>Чт</t>
         </is>
       </c>
-      <c r="BO2" s="7" t="inlineStr">
+      <c r="BO2" s="9" t="inlineStr">
         <is>
           <t>Пт</t>
         </is>
@@ -1604,7 +1626,7 @@
           <t>Пт</t>
         </is>
       </c>
-      <c r="BW2" s="7" t="inlineStr">
+      <c r="BW2" s="9" t="inlineStr">
         <is>
           <t>Сб</t>
         </is>
@@ -1774,7 +1796,7 @@
           <t>Чт</t>
         </is>
       </c>
-      <c r="DE2" s="7" t="inlineStr">
+      <c r="DE2" s="9" t="inlineStr">
         <is>
           <t>Пт</t>
         </is>
@@ -1878,25 +1900,21 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>01.03.2026</t>
+          <t>02.03.2026</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>14.03.2026</t>
+          <t>13.03.2026</t>
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="F3" s="8" t="inlineStr"/>
       <c r="G3" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -1922,16 +1940,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="L3" s="8" t="inlineStr"/>
+      <c r="M3" s="10" t="inlineStr"/>
       <c r="N3" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -1957,11 +1967,7 @@
           <t>■</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="S3" s="8" t="inlineStr"/>
       <c r="T3" s="8" t="inlineStr"/>
       <c r="U3" s="3" t="inlineStr"/>
       <c r="V3" s="3" t="inlineStr"/>
@@ -2009,7 +2015,7 @@
       <c r="BL3" s="3" t="inlineStr"/>
       <c r="BM3" s="3" t="inlineStr"/>
       <c r="BN3" s="3" t="inlineStr"/>
-      <c r="BO3" s="3" t="inlineStr"/>
+      <c r="BO3" s="10" t="inlineStr"/>
       <c r="BP3" s="8" t="inlineStr"/>
       <c r="BQ3" s="8" t="inlineStr"/>
       <c r="BR3" s="3" t="inlineStr"/>
@@ -2017,7 +2023,7 @@
       <c r="BT3" s="3" t="inlineStr"/>
       <c r="BU3" s="3" t="inlineStr"/>
       <c r="BV3" s="3" t="inlineStr"/>
-      <c r="BW3" s="8" t="inlineStr"/>
+      <c r="BW3" s="10" t="inlineStr"/>
       <c r="BX3" s="8" t="inlineStr"/>
       <c r="BY3" s="3" t="inlineStr"/>
       <c r="BZ3" s="3" t="inlineStr"/>
@@ -2051,7 +2057,7 @@
       <c r="DB3" s="3" t="inlineStr"/>
       <c r="DC3" s="3" t="inlineStr"/>
       <c r="DD3" s="3" t="inlineStr"/>
-      <c r="DE3" s="3" t="inlineStr"/>
+      <c r="DE3" s="10" t="inlineStr"/>
       <c r="DF3" s="8" t="inlineStr"/>
       <c r="DG3" s="8" t="inlineStr"/>
       <c r="DH3" s="3" t="inlineStr"/>
@@ -2079,16 +2085,16 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>15.03.2026</t>
+          <t>16.03.2026</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>04.04.2026</t>
+          <t>03.04.2026</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>5</v>
@@ -2100,18 +2106,14 @@
       <c r="J4" s="3" t="inlineStr"/>
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="8" t="inlineStr"/>
-      <c r="M4" s="8" t="inlineStr"/>
+      <c r="M4" s="10" t="inlineStr"/>
       <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="3" t="inlineStr"/>
       <c r="Q4" s="3" t="inlineStr"/>
       <c r="R4" s="3" t="inlineStr"/>
       <c r="S4" s="8" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="T4" s="8" t="inlineStr"/>
       <c r="U4" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2137,16 +2139,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="Z4" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="AA4" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="Z4" s="8" t="inlineStr"/>
+      <c r="AA4" s="8" t="inlineStr"/>
       <c r="AB4" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2172,16 +2166,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="AG4" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="AH4" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="AG4" s="8" t="inlineStr"/>
+      <c r="AH4" s="8" t="inlineStr"/>
       <c r="AI4" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2207,11 +2193,7 @@
           <t>■</t>
         </is>
       </c>
-      <c r="AN4" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="AN4" s="8" t="inlineStr"/>
       <c r="AO4" s="8" t="inlineStr"/>
       <c r="AP4" s="3" t="inlineStr"/>
       <c r="AQ4" s="3" t="inlineStr"/>
@@ -2238,7 +2220,7 @@
       <c r="BL4" s="3" t="inlineStr"/>
       <c r="BM4" s="3" t="inlineStr"/>
       <c r="BN4" s="3" t="inlineStr"/>
-      <c r="BO4" s="3" t="inlineStr"/>
+      <c r="BO4" s="10" t="inlineStr"/>
       <c r="BP4" s="8" t="inlineStr"/>
       <c r="BQ4" s="8" t="inlineStr"/>
       <c r="BR4" s="3" t="inlineStr"/>
@@ -2246,7 +2228,7 @@
       <c r="BT4" s="3" t="inlineStr"/>
       <c r="BU4" s="3" t="inlineStr"/>
       <c r="BV4" s="3" t="inlineStr"/>
-      <c r="BW4" s="8" t="inlineStr"/>
+      <c r="BW4" s="10" t="inlineStr"/>
       <c r="BX4" s="8" t="inlineStr"/>
       <c r="BY4" s="3" t="inlineStr"/>
       <c r="BZ4" s="3" t="inlineStr"/>
@@ -2280,7 +2262,7 @@
       <c r="DB4" s="3" t="inlineStr"/>
       <c r="DC4" s="3" t="inlineStr"/>
       <c r="DD4" s="3" t="inlineStr"/>
-      <c r="DE4" s="3" t="inlineStr"/>
+      <c r="DE4" s="10" t="inlineStr"/>
       <c r="DF4" s="8" t="inlineStr"/>
       <c r="DG4" s="8" t="inlineStr"/>
       <c r="DH4" s="3" t="inlineStr"/>
@@ -2308,16 +2290,16 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>05.04.2026</t>
+          <t>06.04.2026</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>25.04.2026</t>
+          <t>24.04.2026</t>
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>5</v>
@@ -2329,7 +2311,7 @@
       <c r="J5" s="3" t="inlineStr"/>
       <c r="K5" s="3" t="inlineStr"/>
       <c r="L5" s="8" t="inlineStr"/>
-      <c r="M5" s="8" t="inlineStr"/>
+      <c r="M5" s="10" t="inlineStr"/>
       <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr"/>
       <c r="P5" s="3" t="inlineStr"/>
@@ -2357,11 +2339,7 @@
       <c r="AL5" s="3" t="inlineStr"/>
       <c r="AM5" s="3" t="inlineStr"/>
       <c r="AN5" s="8" t="inlineStr"/>
-      <c r="AO5" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="AO5" s="8" t="inlineStr"/>
       <c r="AP5" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2387,16 +2365,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="AU5" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="AV5" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="AU5" s="8" t="inlineStr"/>
+      <c r="AV5" s="8" t="inlineStr"/>
       <c r="AW5" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2422,16 +2392,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="BB5" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="BC5" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="BB5" s="8" t="inlineStr"/>
+      <c r="BC5" s="8" t="inlineStr"/>
       <c r="BD5" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2457,17 +2419,13 @@
           <t>■</t>
         </is>
       </c>
-      <c r="BI5" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="BI5" s="8" t="inlineStr"/>
       <c r="BJ5" s="8" t="inlineStr"/>
       <c r="BK5" s="3" t="inlineStr"/>
       <c r="BL5" s="3" t="inlineStr"/>
       <c r="BM5" s="3" t="inlineStr"/>
       <c r="BN5" s="3" t="inlineStr"/>
-      <c r="BO5" s="3" t="inlineStr"/>
+      <c r="BO5" s="10" t="inlineStr"/>
       <c r="BP5" s="8" t="inlineStr"/>
       <c r="BQ5" s="8" t="inlineStr"/>
       <c r="BR5" s="3" t="inlineStr"/>
@@ -2475,7 +2433,7 @@
       <c r="BT5" s="3" t="inlineStr"/>
       <c r="BU5" s="3" t="inlineStr"/>
       <c r="BV5" s="3" t="inlineStr"/>
-      <c r="BW5" s="8" t="inlineStr"/>
+      <c r="BW5" s="10" t="inlineStr"/>
       <c r="BX5" s="8" t="inlineStr"/>
       <c r="BY5" s="3" t="inlineStr"/>
       <c r="BZ5" s="3" t="inlineStr"/>
@@ -2509,7 +2467,7 @@
       <c r="DB5" s="3" t="inlineStr"/>
       <c r="DC5" s="3" t="inlineStr"/>
       <c r="DD5" s="3" t="inlineStr"/>
-      <c r="DE5" s="3" t="inlineStr"/>
+      <c r="DE5" s="10" t="inlineStr"/>
       <c r="DF5" s="8" t="inlineStr"/>
       <c r="DG5" s="8" t="inlineStr"/>
       <c r="DH5" s="3" t="inlineStr"/>
@@ -2537,16 +2495,16 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>26.04.2026</t>
+          <t>27.04.2026</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>23.05.2026</t>
+          <t>22.05.2026</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>5</v>
@@ -2558,7 +2516,7 @@
       <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="8" t="inlineStr"/>
-      <c r="M6" s="8" t="inlineStr"/>
+      <c r="M6" s="10" t="inlineStr"/>
       <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr"/>
       <c r="P6" s="3" t="inlineStr"/>
@@ -2607,11 +2565,7 @@
       <c r="BG6" s="3" t="inlineStr"/>
       <c r="BH6" s="3" t="inlineStr"/>
       <c r="BI6" s="8" t="inlineStr"/>
-      <c r="BJ6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="BJ6" s="8" t="inlineStr"/>
       <c r="BK6" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2632,21 +2586,9 @@
           <t>■</t>
         </is>
       </c>
-      <c r="BO6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="BP6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="BQ6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="BO6" s="10" t="inlineStr"/>
+      <c r="BP6" s="8" t="inlineStr"/>
+      <c r="BQ6" s="8" t="inlineStr"/>
       <c r="BR6" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2672,16 +2614,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="BW6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="BX6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="BW6" s="10" t="inlineStr"/>
+      <c r="BX6" s="8" t="inlineStr"/>
       <c r="BY6" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2707,16 +2641,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="CD6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="CE6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="CD6" s="8" t="inlineStr"/>
+      <c r="CE6" s="8" t="inlineStr"/>
       <c r="CF6" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2742,11 +2668,7 @@
           <t>■</t>
         </is>
       </c>
-      <c r="CK6" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="CK6" s="8" t="inlineStr"/>
       <c r="CL6" s="8" t="inlineStr"/>
       <c r="CM6" s="3" t="inlineStr"/>
       <c r="CN6" s="3" t="inlineStr"/>
@@ -2766,7 +2688,7 @@
       <c r="DB6" s="3" t="inlineStr"/>
       <c r="DC6" s="3" t="inlineStr"/>
       <c r="DD6" s="3" t="inlineStr"/>
-      <c r="DE6" s="3" t="inlineStr"/>
+      <c r="DE6" s="10" t="inlineStr"/>
       <c r="DF6" s="8" t="inlineStr"/>
       <c r="DG6" s="8" t="inlineStr"/>
       <c r="DH6" s="3" t="inlineStr"/>
@@ -2794,16 +2716,16 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>24.05.2026</t>
+          <t>25.05.2026</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>13.06.2026</t>
+          <t>16.06.2026</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>5</v>
@@ -2815,7 +2737,7 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="8" t="inlineStr"/>
-      <c r="M7" s="8" t="inlineStr"/>
+      <c r="M7" s="10" t="inlineStr"/>
       <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr"/>
       <c r="P7" s="3" t="inlineStr"/>
@@ -2869,7 +2791,7 @@
       <c r="BL7" s="3" t="inlineStr"/>
       <c r="BM7" s="3" t="inlineStr"/>
       <c r="BN7" s="3" t="inlineStr"/>
-      <c r="BO7" s="3" t="inlineStr"/>
+      <c r="BO7" s="10" t="inlineStr"/>
       <c r="BP7" s="8" t="inlineStr"/>
       <c r="BQ7" s="8" t="inlineStr"/>
       <c r="BR7" s="3" t="inlineStr"/>
@@ -2877,7 +2799,7 @@
       <c r="BT7" s="3" t="inlineStr"/>
       <c r="BU7" s="3" t="inlineStr"/>
       <c r="BV7" s="3" t="inlineStr"/>
-      <c r="BW7" s="8" t="inlineStr"/>
+      <c r="BW7" s="10" t="inlineStr"/>
       <c r="BX7" s="8" t="inlineStr"/>
       <c r="BY7" s="3" t="inlineStr"/>
       <c r="BZ7" s="3" t="inlineStr"/>
@@ -2892,11 +2814,7 @@
       <c r="CI7" s="3" t="inlineStr"/>
       <c r="CJ7" s="3" t="inlineStr"/>
       <c r="CK7" s="8" t="inlineStr"/>
-      <c r="CL7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="CL7" s="8" t="inlineStr"/>
       <c r="CM7" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2922,16 +2840,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="CR7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="CS7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="CR7" s="8" t="inlineStr"/>
+      <c r="CS7" s="8" t="inlineStr"/>
       <c r="CT7" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2957,16 +2867,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="CY7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="CZ7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="CY7" s="8" t="inlineStr"/>
+      <c r="CZ7" s="8" t="inlineStr"/>
       <c r="DA7" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -2987,19 +2889,19 @@
           <t>■</t>
         </is>
       </c>
-      <c r="DE7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DF7" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="DE7" s="10" t="inlineStr"/>
+      <c r="DF7" s="8" t="inlineStr"/>
       <c r="DG7" s="8" t="inlineStr"/>
-      <c r="DH7" s="3" t="inlineStr"/>
-      <c r="DI7" s="3" t="inlineStr"/>
+      <c r="DH7" s="4" t="inlineStr">
+        <is>
+          <t>■</t>
+        </is>
+      </c>
+      <c r="DI7" s="4" t="inlineStr">
+        <is>
+          <t>■</t>
+        </is>
+      </c>
       <c r="DJ7" s="3" t="inlineStr"/>
       <c r="DK7" s="3" t="inlineStr"/>
       <c r="DL7" s="3" t="inlineStr"/>
@@ -3023,16 +2925,16 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>14.06.2026</t>
+          <t>17.06.2026</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>27.06.2026</t>
+          <t>24.06.2026</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>5</v>
@@ -3044,7 +2946,7 @@
       <c r="J8" s="3" t="inlineStr"/>
       <c r="K8" s="3" t="inlineStr"/>
       <c r="L8" s="8" t="inlineStr"/>
-      <c r="M8" s="8" t="inlineStr"/>
+      <c r="M8" s="10" t="inlineStr"/>
       <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr"/>
@@ -3098,7 +3000,7 @@
       <c r="BL8" s="3" t="inlineStr"/>
       <c r="BM8" s="3" t="inlineStr"/>
       <c r="BN8" s="3" t="inlineStr"/>
-      <c r="BO8" s="3" t="inlineStr"/>
+      <c r="BO8" s="10" t="inlineStr"/>
       <c r="BP8" s="8" t="inlineStr"/>
       <c r="BQ8" s="8" t="inlineStr"/>
       <c r="BR8" s="3" t="inlineStr"/>
@@ -3106,7 +3008,7 @@
       <c r="BT8" s="3" t="inlineStr"/>
       <c r="BU8" s="3" t="inlineStr"/>
       <c r="BV8" s="3" t="inlineStr"/>
-      <c r="BW8" s="8" t="inlineStr"/>
+      <c r="BW8" s="10" t="inlineStr"/>
       <c r="BX8" s="8" t="inlineStr"/>
       <c r="BY8" s="3" t="inlineStr"/>
       <c r="BZ8" s="3" t="inlineStr"/>
@@ -3140,23 +3042,11 @@
       <c r="DB8" s="3" t="inlineStr"/>
       <c r="DC8" s="3" t="inlineStr"/>
       <c r="DD8" s="3" t="inlineStr"/>
-      <c r="DE8" s="3" t="inlineStr"/>
+      <c r="DE8" s="10" t="inlineStr"/>
       <c r="DF8" s="8" t="inlineStr"/>
-      <c r="DG8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DH8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DI8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="DG8" s="8" t="inlineStr"/>
+      <c r="DH8" s="3" t="inlineStr"/>
+      <c r="DI8" s="3" t="inlineStr"/>
       <c r="DJ8" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -3172,16 +3062,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="DM8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DN8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="DM8" s="8" t="inlineStr"/>
+      <c r="DN8" s="8" t="inlineStr"/>
       <c r="DO8" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -3197,21 +3079,9 @@
           <t>■</t>
         </is>
       </c>
-      <c r="DR8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DS8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DT8" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="DR8" s="3" t="inlineStr"/>
+      <c r="DS8" s="3" t="inlineStr"/>
+      <c r="DT8" s="8" t="inlineStr"/>
       <c r="DU8" s="8" t="inlineStr"/>
       <c r="DV8" s="3" t="inlineStr"/>
       <c r="DW8" s="3" t="inlineStr"/>
@@ -3224,7 +3094,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>21.06.2026</t>
+          <t>25.06.2026</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -3233,7 +3103,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>5</v>
@@ -3245,7 +3115,7 @@
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr"/>
       <c r="L9" s="8" t="inlineStr"/>
-      <c r="M9" s="8" t="inlineStr"/>
+      <c r="M9" s="10" t="inlineStr"/>
       <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr"/>
       <c r="P9" s="3" t="inlineStr"/>
@@ -3299,7 +3169,7 @@
       <c r="BL9" s="3" t="inlineStr"/>
       <c r="BM9" s="3" t="inlineStr"/>
       <c r="BN9" s="3" t="inlineStr"/>
-      <c r="BO9" s="3" t="inlineStr"/>
+      <c r="BO9" s="10" t="inlineStr"/>
       <c r="BP9" s="8" t="inlineStr"/>
       <c r="BQ9" s="8" t="inlineStr"/>
       <c r="BR9" s="3" t="inlineStr"/>
@@ -3307,7 +3177,7 @@
       <c r="BT9" s="3" t="inlineStr"/>
       <c r="BU9" s="3" t="inlineStr"/>
       <c r="BV9" s="3" t="inlineStr"/>
-      <c r="BW9" s="8" t="inlineStr"/>
+      <c r="BW9" s="10" t="inlineStr"/>
       <c r="BX9" s="8" t="inlineStr"/>
       <c r="BY9" s="3" t="inlineStr"/>
       <c r="BZ9" s="3" t="inlineStr"/>
@@ -3341,7 +3211,7 @@
       <c r="DB9" s="3" t="inlineStr"/>
       <c r="DC9" s="3" t="inlineStr"/>
       <c r="DD9" s="3" t="inlineStr"/>
-      <c r="DE9" s="3" t="inlineStr"/>
+      <c r="DE9" s="10" t="inlineStr"/>
       <c r="DF9" s="8" t="inlineStr"/>
       <c r="DG9" s="8" t="inlineStr"/>
       <c r="DH9" s="3" t="inlineStr"/>
@@ -3350,26 +3220,10 @@
       <c r="DK9" s="3" t="inlineStr"/>
       <c r="DL9" s="3" t="inlineStr"/>
       <c r="DM9" s="8" t="inlineStr"/>
-      <c r="DN9" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DO9" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DP9" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DQ9" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="DN9" s="8" t="inlineStr"/>
+      <c r="DO9" s="3" t="inlineStr"/>
+      <c r="DP9" s="3" t="inlineStr"/>
+      <c r="DQ9" s="3" t="inlineStr"/>
       <c r="DR9" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -3380,16 +3234,8 @@
           <t>■</t>
         </is>
       </c>
-      <c r="DT9" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
-      <c r="DU9" s="4" t="inlineStr">
-        <is>
-          <t>■</t>
-        </is>
-      </c>
+      <c r="DT9" s="8" t="inlineStr"/>
+      <c r="DU9" s="8" t="inlineStr"/>
       <c r="DV9" s="4" t="inlineStr">
         <is>
           <t>■</t>
@@ -3398,6 +3244,76 @@
       <c r="DW9" s="4" t="inlineStr">
         <is>
           <t>■</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Легенда цветов</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Зеленый</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Рабочий день выполнения этапа</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Серый</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Выходной (суббота/воскресенье)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Красный</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Праздничный нерабочий день</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Праздничные дни (без учета переносов):</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>08.03, 01.05, 09.05, 12.06</t>
         </is>
       </c>
     </row>

</xml_diff>